<commit_message>
chore(catalog): update affiliate-partners.xlsx for 2026-06-28 sync
Sets Last Updated=2026-06-28 and per-brand Notes for the 7 active
brands (ENGWE, Eunorau, Walfiske, DUOTTS, SAMEBIKE, Dyucycle,
vtuviabike). Was skipped during the weekly sync run because Excel
had the file open (PermissionError).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Fatbikes, folding e-bikes</t>
+          <t>+4 new (L16, Y400, Ease 2 Pro, Y600). 10 price changes flagged for review (price_usd was NULL, currency uncertain).</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>US-based, multiple dealers</t>
+          <t>+8 new (S1, FAT-HD 1.0, FAT-HD 2.0, SPECTER-S 3.0, SPECTER-ST 2.0, FAT-HS, E-FAT-MN, MAX-CARGO 2.0). 7 price updates applied.</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Online only, no physical stores</t>
+          <t>No changes applied. 1 fuzzy price match flagged for review (ET-7 Ultra vs vendor motor variant).</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>Online only, no physical stores. 6 new models added.</t>
+          <t>11 price updates applied (range -$200 to +$70).</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>Online only + Walmart. 19 models added.</t>
+          <t>+3 new (STORM, CREST, RS-A08-II). 17 price updates applied (~10% drops).</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>Online only. 7 models added as brand DYU.</t>
+          <t>+3 new (C6, C2, C5) inserted as brand DYU. 7 price updates applied.</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>US-based brand. 8 models added. Online only.</t>
+          <t>+3 new (FMB, Giraffe, Reindeer 1.0) inserted as brand VTUVIA. 1 price change flagged: CMB $2149 is new 10-speed variant, not a price change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalog): weekly sync - 2 price drops applied (R1+, WF26)
Re-scraped active affiliate brands (ENGWE, Eunorau, Walfiske, DUOTTS,
SAMEBIKE, DYU, VTUVIA). Applied only the two cleanest signals:

- Eunorau R1+ (eunorau-r1-plus): $4999.00 -> $4499.00 (-$500.00)
- Walfiske WF26: $1199.00 -> $999.00 (-$200.00)

All other findings deferred for owner review (see CATALOG-SYNC-LOG.md):
- ENGWE vendor catalog underwent a generation rotation (L20/M20/EP-2
  multi-version SKUs, new Ease 1/3, X20/X26 split, 9 likely-discontinued)
- Eunorau FLASH 2.0 vendor price reverted last week's drop, R1 Compact
  is a new SKU candidate
- Walfiske ET-7 Ultra has 3 vendor variants at different prices now
- DUOTTS, SAMEBIKE, VTUVIA only had matcher false positives (UK variants,
  color variants, 2-char model codes)

affiliate-partners.xlsx Last Updated set to 2026-06-30 for all 7 brands.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>+4 new (L16, Y400, Ease 2 Pro, Y600). 10 price changes flagged for review (price_usd was NULL, currency uncertain).</t>
+          <t>12 price-change candidates flagged for review (vendor catalog underwent generation update: L20/L20 3.0, M20/M20 2.0/M20 3.0, Ease 1/2/3 lines added). 9 possibly-discontinued (P275 Pro/SE/ST, N1 Air/Pro, M1, P20, L20 Boost, Engine X) - none in vendor catalog, left active pending owner review.</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>+8 new (S1, FAT-HD 1.0, FAT-HD 2.0, SPECTER-S 3.0, SPECTER-ST 2.0, FAT-HS, E-FAT-MN, MAX-CARGO 2.0). 7 price updates applied.</t>
+          <t>1 price update applied: R1+ $4999-&gt;$4499. FLASH 2.0 vendor now $2499 (DB $2099 from last week) - deferred, possible vendor revert.</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>No changes applied. 1 fuzzy price match flagged for review (ET-7 Ultra vs vendor motor variant).</t>
+          <t>1 price update applied: WF26 $1199-&gt;$999. ET-7 Ultra has 3 vendor variants now at $2299-$2499, deferred.</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>11 price updates applied (range -$200 to +$70).</t>
+          <t>No changes. Vendor added Ship-to-UK variants and Pre-Owned listing (skipped, not US-market).</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>+3 new (STORM, CREST, RS-A08-II). 17 price updates applied (~10% drops).</t>
+          <t>No changes. Matcher swap noise on CY20/CY20 Pro and RS-A01 MEN/Plus - DB values verified correct.</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>+3 new (C6, C2, C5) inserted as brand DYU. 7 price updates applied.</t>
+          <t>No changes. All 10 DYU bikes still in vendor catalog at unchanged prices.</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>+3 new (FMB, Giraffe, Reindeer 1.0) inserted as brand VTUVIA. 1 price change flagged: CMB $2149 is new 10-speed variant, not a price change.</t>
+          <t>No changes. Vendor lists SX20 and SF20H color variants separately (already represented by single DB rows). CMB 10-speed variant still pending owner decision from last week.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalog): weekly sync - 12 price updates, 10 discontinued marks
Applied the confident findings from the 2026-07-06 weekly sync:

- 12 price updates across ENGWE (8), Eunorau (2), Walfisk (1), DYU (1),
  all matched to vendor by exact handle or high-score suffix/token overlap.
  ENGWE rows also had price_usd populated (was NULL).
- 10 bikes marked available=false after 2+ cycles of confirmed absence
  from vendor catalog: 9 ENGWE (Engine X, L20 Boost, M1, N1 Air, N1 Pro,
  P20, P275 Pro/SE/ST) and SAMEBIKE YINYU14. Product pages stay live
  and switch to the No longer available template.

Deferred: 9 ENGWE NEW candidates (Ease 1/3, M20/L20/X-family new gens),
3 Eunorau NEW candidates (R1 Compact, ICEX, JUMBO), 3 DYU NEW candidates,
9 VTUVIA color variants, and all matcher-noise discontinued flags. See
harkuhh/CATALOG-SYNC-LOG.md for the full breakdown.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>12 price-change candidates flagged for review (vendor catalog underwent generation update: L20/L20 3.0, M20/M20 2.0/M20 3.0, Ease 1/2/3 lines added). 9 possibly-discontinued (P275 Pro/SE/ST, N1 Air/Pro, M1, P20, L20 Boost, Engine X) - none in vendor catalog, left active pending owner review.</t>
+          <t>+0 new, 8 price updates, 9 discontinued (auto: 2+ cycles absent)</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>1 price update applied: R1+ $4999-&gt;$4499. FLASH 2.0 vendor now $2499 (DB $2099 from last week) - deferred, possible vendor revert.</t>
+          <t>+0 new, 2 price updates (FLASH +400, R1 +550), 0 discontinued</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>1 price update applied: WF26 $1199-&gt;$999. ET-7 Ultra has 3 vendor variants now at $2299-$2499, deferred.</t>
+          <t>+0 new, 1 price update (WF26 +200), 0 discontinued</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>No changes. Vendor added Ship-to-UK variants and Pre-Owned listing (skipped, not US-market).</t>
+          <t>clean - all 11 rows match vendor 1:1</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>No changes. Matcher swap noise on CY20/CY20 Pro and RS-A01 MEN/Plus - DB values verified correct.</t>
+          <t>+0 new, 0 price updates, 1 discontinued (YINYU14 - 2 cycles absent)</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>No changes. All 10 DYU bikes still in vendor catalog at unchanged prices.</t>
+          <t>+0 new, 1 price update (D3F +50), 0 discontinued</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>No changes. Vendor lists SX20 and SF20H color variants separately (already represented by single DB rows). CMB 10-speed variant still pending owner decision from last week.</t>
+          <t>+0 new, 0 price updates, 0 discontinued</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalog): weekly sync 2026-07-13 -- 18 price updates, 1 discontinued
Applied 18 vendor price changes across ENGWE, Eunorau, Walfisk, DUOTTS
and SAMEBIKE (all with match score >= 80 and pct delta <= 30%). Marked
Eunorau Defender-S available=false after 2 consecutive cycles absent.
Deferred 30 NEW candidates (mostly ENGWE generational rollover, VTUVIA
color variants, Eunorau accessories) and 6 possibly-discontinued ENGWE
rows pending owner review of the model-line rename.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>+0 new, 8 price updates, 9 discontinued (auto: 2+ cycles absent)</t>
+          <t>2 price updates; 8 new + 6 disc deferred (rollover)</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>+0 new, 2 price updates (FLASH +400, R1 +550), 0 discontinued</t>
+          <t>5 price updates; 1 discontinued; 8 new deferred</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>+0 new, 1 price update (WF26 +200), 0 discontinued</t>
+          <t>1 price update; 3 new deferred; ET-7 Ultra recurring false-match</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>clean - all 11 rows match vendor 1:1</t>
+          <t>9 price updates (broad price cut across line)</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>+0 new, 0 price updates, 1 discontinued (YINYU14 - 2 cycles absent)</t>
+          <t>1 price update; catalog otherwise clean</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>+0 new, 1 price update (D3F +50), 0 discontinued</t>
+          <t>2 new deferred; A1F Pro price ambiguous</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>+0 new, 0 price updates, 0 discontinued</t>
+          <t>9 color/variant duplicates skipped; catalog stable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalog): weekly sync (run 39) - 4 price updates, 21 items deferred
SAMEBIKE: M20 $1429 -> $1299; M20-III $1749 -> $1599.
DYU: M20 $949 -> $899; D3F $549 -> $499.

Deferred (owner review): ENGWE 12 new + 5 disc (4th cycle vendor rollover),
Eunorau R1 rename to R1-19 (-$549), Walfisk ET-7 Ultra recurring false-match,
DYU A1F Pro ambiguous, VTUVIA 11 color/variant duplicates.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructies" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Affiliate Partners'!$A$1:$L$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Affiliate Partners'!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2 price updates; 8 new + 6 disc deferred (rollover)</t>
+          <t>0 changes; 12 rollover new + 5 disc deferred (recurring)</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>5 price updates; 1 discontinued; 8 new deferred</t>
+          <t>0 applied; R1 rename to R1-19 -$549 deferred; 4 new deferred</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>1 price update; 3 new deferred; ET-7 Ultra recurring false-match</t>
+          <t>0 applied; ET-7 Ultra recurring false-match deferred</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>9 price updates (broad price cut across line)</t>
+          <t>clean (11 unchanged, no changes)</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>1 price update; catalog otherwise clean</t>
+          <t>2 price updates (M20 -$130, M20-III -$150)</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>2 new deferred; A1F Pro price ambiguous</t>
+          <t>2 price updates (M20 -$50, D3F -$50); A1F Pro ambiguous deferred</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>9 color/variant duplicates skipped; catalog stable</t>
+          <t>0 applied; color-variant duplicates and 3 new (Gemini, CMB, SN100 variants) deferred</t>
         </is>
       </c>
     </row>
@@ -1377,8 +1377,432 @@
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="5" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Amazon Associates</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>https://affiliate-program.amazon.com</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>RETAILER/NETWORK - not a bike brand, skip in /sync-brands. Low commission (~3%) but high conversion; covers brands without their own program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>CJ Affiliate</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cj.com/publishers</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>CJ</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>NETWORK - not a bike brand, skip in /sync-brands. Apply per merchant after account approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Awin</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.awin.com</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Awin</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>NETWORK - not a bike brand, skip in /sync-brands. Refundable signup deposit; per-merchant approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>eBay Partner Network</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>https://partnernetwork.ebay.com</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>eBay</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>NETWORK - not a bike brand, skip in /sync-brands. Strong for refurbished/discontinued models (long-tail search).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>REI</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rei.com</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Check on signup</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>RETAILER (multi-brand) - not a bike brand, skip in /sync-brands. Confirm network at signup. High US brand authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Best Buy</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bestbuy.com</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Check on signup</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>RETAILER (multi-brand) - not a bike brand, skip in /sync-brands. Confirm network at signup. Broad mainstream selection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.walmart.com</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Check on signup</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>RETAILER (multi-brand) - not a bike brand, skip in /sync-brands. Confirm network at signup. Covers budget segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Backcountry</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.backcountry.com</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Check on signup</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>RETAILER (multi-brand) - not a bike brand, skip in /sync-brands. Confirm network at signup. Premium/outdoor positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Skimlinks</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>https://skimlinks.com</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Skimlinks</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>FALLBACK NETWORK - not a bike brand, skip in /sync-brands. Auto-converts links to merchants without a direct deal. Lower margin, monetises the rest of the catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sovrn Commerce</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sovrn.com/commerce</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Sovrn</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>FALLBACK NETWORK - not a bike brand, skip in /sync-brands. Alternative to Skimlinks; compare terms before choosing one.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L19"/>
+  <autoFilter ref="A1:L29"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
@@ -1394,7 +1818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -1578,14 +2002,14 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Bikes Scraped      = Yes/No - zijn de fietsen al gescraped?</t>
+          <t xml:space="preserve">  Bikes Scraped      = Yes/No - zijn de fietsen al gescraped? (N/A = retailer/netwerk, niet scrapen)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stores Scraped     = Yes/No - zijn de stores al gescraped?</t>
+          <t xml:space="preserve">  Stores Scraped     = Yes/No - zijn de stores al gescraped? (N/A = retailer/netwerk, niet scrapen)</t>
         </is>
       </c>
     </row>
@@ -1600,6 +2024,20 @@
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  Notes              = Extra opmerkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>LET OP: rijen met N/A in Bikes/Stores Scraped zijn retailers of netwerken,</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>geen fietsmerken. /sync-brands moet deze overslaan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalog): weekly sync (2026-07-29) -- 2 price updates, no new/disc
- ENGWE L16 $899 -> $849 (exact-handle match, clean $50 markdown)
- Eunorau R1 $4299 -> $3750 (R1-19 rename applied 3rd cycle, exact-handle
  match, -12.8% within auto-apply threshold)

DB rows synced live via Supabase. 21 SAMEBIKE, 9 DYU, 3 Walfisk, 11 DUOTTS,
11 VTUVIA and 24 Eunorau rows unchanged. ENGWE rollover (5th cycle) still
deferred pending owner sign-off: 2 price defers, 7 new candidates, 3
possibly-discontinued rows. See CATALOG-SYNC-LOG.md for the full breakdown.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/harkuhh/affiliate-partners.xlsx
+++ b/harkuhh/affiliate-partners.xlsx
@@ -654,12 +654,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>0 changes; 12 rollover new + 5 disc deferred (recurring)</t>
+          <t>1 price (L16 -$50); rollover new/disc still deferred (5th cycle)</t>
         </is>
       </c>
     </row>
@@ -708,12 +708,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>0 applied; R1 rename to R1-19 -$549 deferred; 4 new deferred</t>
+          <t>1 price (R1 -$549, R1-19 rename 3rd-cycle apply); META275 dup + 4 new deferred</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>0 applied; ET-7 Ultra recurring false-match deferred</t>
+          <t>clean (3 unchanged)</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>clean (11 unchanged, no changes)</t>
+          <t>clean (11 unchanged)</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>2 price updates (M20 -$130, M20-III -$150)</t>
+          <t>clean (21/22 matched, no changes)</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L15" s="21" t="inlineStr">
         <is>
-          <t>2 price updates (M20 -$50, D3F -$50); A1F Pro ambiguous deferred</t>
+          <t>clean (9/10 matched); A1F Pro price ambiguous deferred</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>0 applied; color-variant duplicates and 3 new (Gemini, CMB, SN100 variants) deferred</t>
+          <t>clean (11 unchanged); 9 color-variant duplicates deferred</t>
         </is>
       </c>
     </row>

</xml_diff>